<commit_message>
feat: add Ikun boss and basketball prop
</commit_message>
<xml_diff>
--- a/LubanData/Data/#game.Enemy.xlsx
+++ b/LubanData/Data/#game.Enemy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2d0407bc9e6b490e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R53d14db3583d4eb2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -584,6 +584,33 @@
         <x:v>公鸡敌人</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8"/>
+      <x:c r="B8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Ikun</x:v>
+      </x:c>
+      <x:c r="D8" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>ikun Boss</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>